<commit_message>
Adding burst screen capture to improve killfeed detection
</commit_message>
<xml_diff>
--- a/ow_coach_ai_annotation_template.xlsx
+++ b/ow_coach_ai_annotation_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b2cb65643c67e91f/Desktop/Coding/ow_coach/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="685" documentId="11_5BD94D31B6F49361A4904CBFDA1A4848FA157360" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B25A5E81-5565-4A59-BEED-F048E3E34F7E}"/>
+  <xr:revisionPtr revIDLastSave="686" documentId="11_5BD94D31B6F49361A4904CBFDA1A4848FA157360" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5F7881BC-1536-4E47-97AE-4D5DE68C0C22}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="21840" windowHeight="37920" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -282,7 +282,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1031" uniqueCount="235">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1032" uniqueCount="236">
   <si>
     <t>OW Coach AI Annotation Workbook</t>
   </si>
@@ -988,6 +988,9 @@
   <si>
     <t>The ult % of 42 is for Zen</t>
   </si>
+  <si>
+    <t>707 to 721</t>
+  </si>
 </sst>
 </file>
 
@@ -7163,97 +7166,100 @@
       <c r="S112" s="8"/>
       <c r="V112" s="9"/>
     </row>
-    <row r="113" spans="16:22" x14ac:dyDescent="0.25">
+    <row r="113" spans="3:22" x14ac:dyDescent="0.25">
       <c r="P113" s="8"/>
       <c r="Q113" s="8"/>
       <c r="S113" s="8"/>
       <c r="V113" s="9"/>
     </row>
-    <row r="114" spans="16:22" x14ac:dyDescent="0.25">
+    <row r="114" spans="3:22" x14ac:dyDescent="0.25">
       <c r="P114" s="8"/>
       <c r="Q114" s="8"/>
       <c r="S114" s="8"/>
       <c r="V114" s="9"/>
     </row>
-    <row r="115" spans="16:22" x14ac:dyDescent="0.25">
+    <row r="115" spans="3:22" x14ac:dyDescent="0.25">
+      <c r="C115" t="s">
+        <v>235</v>
+      </c>
       <c r="P115" s="8"/>
       <c r="Q115" s="8"/>
       <c r="S115" s="8"/>
       <c r="V115" s="9"/>
     </row>
-    <row r="116" spans="16:22" x14ac:dyDescent="0.25">
+    <row r="116" spans="3:22" x14ac:dyDescent="0.25">
       <c r="P116" s="8"/>
       <c r="Q116" s="8"/>
       <c r="S116" s="8"/>
       <c r="V116" s="9"/>
     </row>
-    <row r="117" spans="16:22" x14ac:dyDescent="0.25">
+    <row r="117" spans="3:22" x14ac:dyDescent="0.25">
       <c r="P117" s="8"/>
       <c r="Q117" s="8"/>
       <c r="S117" s="8"/>
       <c r="V117" s="9"/>
     </row>
-    <row r="118" spans="16:22" x14ac:dyDescent="0.25">
+    <row r="118" spans="3:22" x14ac:dyDescent="0.25">
       <c r="P118" s="8"/>
       <c r="Q118" s="8"/>
       <c r="S118" s="8"/>
       <c r="V118" s="9"/>
     </row>
-    <row r="119" spans="16:22" x14ac:dyDescent="0.25">
+    <row r="119" spans="3:22" x14ac:dyDescent="0.25">
       <c r="P119" s="8"/>
       <c r="Q119" s="8"/>
       <c r="S119" s="8"/>
       <c r="V119" s="9"/>
     </row>
-    <row r="120" spans="16:22" x14ac:dyDescent="0.25">
+    <row r="120" spans="3:22" x14ac:dyDescent="0.25">
       <c r="P120" s="8"/>
       <c r="Q120" s="8"/>
       <c r="S120" s="8"/>
       <c r="V120" s="9"/>
     </row>
-    <row r="121" spans="16:22" x14ac:dyDescent="0.25">
+    <row r="121" spans="3:22" x14ac:dyDescent="0.25">
       <c r="P121" s="8"/>
       <c r="Q121" s="8"/>
       <c r="S121" s="8"/>
       <c r="V121" s="9"/>
     </row>
-    <row r="122" spans="16:22" x14ac:dyDescent="0.25">
+    <row r="122" spans="3:22" x14ac:dyDescent="0.25">
       <c r="P122" s="8"/>
       <c r="Q122" s="8"/>
       <c r="S122" s="8"/>
       <c r="V122" s="9"/>
     </row>
-    <row r="123" spans="16:22" x14ac:dyDescent="0.25">
+    <row r="123" spans="3:22" x14ac:dyDescent="0.25">
       <c r="P123" s="8"/>
       <c r="Q123" s="8"/>
       <c r="S123" s="8"/>
       <c r="V123" s="9"/>
     </row>
-    <row r="124" spans="16:22" x14ac:dyDescent="0.25">
+    <row r="124" spans="3:22" x14ac:dyDescent="0.25">
       <c r="P124" s="8"/>
       <c r="Q124" s="8"/>
       <c r="S124" s="8"/>
       <c r="V124" s="9"/>
     </row>
-    <row r="125" spans="16:22" x14ac:dyDescent="0.25">
+    <row r="125" spans="3:22" x14ac:dyDescent="0.25">
       <c r="P125" s="8"/>
       <c r="Q125" s="8"/>
       <c r="S125" s="8"/>
       <c r="V125" s="9"/>
     </row>
-    <row r="126" spans="16:22" x14ac:dyDescent="0.25">
+    <row r="126" spans="3:22" x14ac:dyDescent="0.25">
       <c r="P126" s="8"/>
       <c r="Q126" s="8"/>
       <c r="S126" s="8"/>
       <c r="V126" s="9"/>
     </row>
-    <row r="127" spans="16:22" x14ac:dyDescent="0.25">
+    <row r="127" spans="3:22" x14ac:dyDescent="0.25">
       <c r="P127" s="8"/>
       <c r="Q127" s="8"/>
       <c r="S127" s="8"/>
       <c r="V127" s="9"/>
     </row>
-    <row r="128" spans="16:22" x14ac:dyDescent="0.25">
+    <row r="128" spans="3:22" x14ac:dyDescent="0.25">
       <c r="P128" s="8"/>
       <c r="Q128" s="8"/>
       <c r="S128" s="8"/>

</xml_diff>

<commit_message>
Rolled back ROI cross-section to previous param to reduce clutter
</commit_message>
<xml_diff>
--- a/ow_coach_ai_annotation_template.xlsx
+++ b/ow_coach_ai_annotation_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b2cb65643c67e91f/Desktop/Coding/ow_coach/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="686" documentId="11_5BD94D31B6F49361A4904CBFDA1A4848FA157360" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5F7881BC-1536-4E47-97AE-4D5DE68C0C22}"/>
+  <xr:revisionPtr revIDLastSave="687" documentId="11_5BD94D31B6F49361A4904CBFDA1A4848FA157360" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{70107B1E-A307-4CC4-B064-C57BAE3AF756}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="-120" windowWidth="21840" windowHeight="37920" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -282,7 +282,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1032" uniqueCount="236">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1033" uniqueCount="237">
   <si>
     <t>OW Coach AI Annotation Workbook</t>
   </si>
@@ -991,6 +991,209 @@
   <si>
     <t>707 to 721</t>
   </si>
+  <si>
+    <r>
+      <t xml:space="preserve">    </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF9CDCFE"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>killfeed_roi</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve">: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4EC9B0"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>tuple</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>[</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4EC9B0"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>float</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4EC9B0"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>float</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4EC9B0"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>float</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4EC9B0"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>float</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve">] </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFD4D4D4"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>=</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> (</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFB5CEA8"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>0.8</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFB5CEA8"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>0.15</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFB5CEA8"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>0.985</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFB5CEA8"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>0.185</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>)</t>
+    </r>
+  </si>
 </sst>
 </file>
 
@@ -1000,7 +1203,7 @@
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="167" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
   </numFmts>
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1053,6 +1256,36 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFCCCCCC"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9CDCFE"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF4EC9B0"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFD4D4D4"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFB5CEA8"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -1098,7 +1331,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1132,6 +1365,9 @@
     <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -7166,19 +7402,19 @@
       <c r="S112" s="8"/>
       <c r="V112" s="9"/>
     </row>
-    <row r="113" spans="3:22" x14ac:dyDescent="0.25">
+    <row r="113" spans="2:22" x14ac:dyDescent="0.25">
       <c r="P113" s="8"/>
       <c r="Q113" s="8"/>
       <c r="S113" s="8"/>
       <c r="V113" s="9"/>
     </row>
-    <row r="114" spans="3:22" x14ac:dyDescent="0.25">
+    <row r="114" spans="2:22" x14ac:dyDescent="0.25">
       <c r="P114" s="8"/>
       <c r="Q114" s="8"/>
       <c r="S114" s="8"/>
       <c r="V114" s="9"/>
     </row>
-    <row r="115" spans="3:22" x14ac:dyDescent="0.25">
+    <row r="115" spans="2:22" x14ac:dyDescent="0.25">
       <c r="C115" t="s">
         <v>235</v>
       </c>
@@ -7187,79 +7423,82 @@
       <c r="S115" s="8"/>
       <c r="V115" s="9"/>
     </row>
-    <row r="116" spans="3:22" x14ac:dyDescent="0.25">
+    <row r="116" spans="2:22" x14ac:dyDescent="0.25">
       <c r="P116" s="8"/>
       <c r="Q116" s="8"/>
       <c r="S116" s="8"/>
       <c r="V116" s="9"/>
     </row>
-    <row r="117" spans="3:22" x14ac:dyDescent="0.25">
+    <row r="117" spans="2:22" x14ac:dyDescent="0.25">
       <c r="P117" s="8"/>
       <c r="Q117" s="8"/>
       <c r="S117" s="8"/>
       <c r="V117" s="9"/>
     </row>
-    <row r="118" spans="3:22" x14ac:dyDescent="0.25">
+    <row r="118" spans="2:22" x14ac:dyDescent="0.25">
       <c r="P118" s="8"/>
       <c r="Q118" s="8"/>
       <c r="S118" s="8"/>
       <c r="V118" s="9"/>
     </row>
-    <row r="119" spans="3:22" x14ac:dyDescent="0.25">
+    <row r="119" spans="2:22" x14ac:dyDescent="0.25">
       <c r="P119" s="8"/>
       <c r="Q119" s="8"/>
       <c r="S119" s="8"/>
       <c r="V119" s="9"/>
     </row>
-    <row r="120" spans="3:22" x14ac:dyDescent="0.25">
+    <row r="120" spans="2:22" x14ac:dyDescent="0.25">
       <c r="P120" s="8"/>
       <c r="Q120" s="8"/>
       <c r="S120" s="8"/>
       <c r="V120" s="9"/>
     </row>
-    <row r="121" spans="3:22" x14ac:dyDescent="0.25">
+    <row r="121" spans="2:22" x14ac:dyDescent="0.25">
       <c r="P121" s="8"/>
       <c r="Q121" s="8"/>
       <c r="S121" s="8"/>
       <c r="V121" s="9"/>
     </row>
-    <row r="122" spans="3:22" x14ac:dyDescent="0.25">
+    <row r="122" spans="2:22" x14ac:dyDescent="0.25">
       <c r="P122" s="8"/>
       <c r="Q122" s="8"/>
       <c r="S122" s="8"/>
       <c r="V122" s="9"/>
     </row>
-    <row r="123" spans="3:22" x14ac:dyDescent="0.25">
+    <row r="123" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B123" s="18" t="s">
+        <v>236</v>
+      </c>
       <c r="P123" s="8"/>
       <c r="Q123" s="8"/>
       <c r="S123" s="8"/>
       <c r="V123" s="9"/>
     </row>
-    <row r="124" spans="3:22" x14ac:dyDescent="0.25">
+    <row r="124" spans="2:22" x14ac:dyDescent="0.25">
       <c r="P124" s="8"/>
       <c r="Q124" s="8"/>
       <c r="S124" s="8"/>
       <c r="V124" s="9"/>
     </row>
-    <row r="125" spans="3:22" x14ac:dyDescent="0.25">
+    <row r="125" spans="2:22" x14ac:dyDescent="0.25">
       <c r="P125" s="8"/>
       <c r="Q125" s="8"/>
       <c r="S125" s="8"/>
       <c r="V125" s="9"/>
     </row>
-    <row r="126" spans="3:22" x14ac:dyDescent="0.25">
+    <row r="126" spans="2:22" x14ac:dyDescent="0.25">
       <c r="P126" s="8"/>
       <c r="Q126" s="8"/>
       <c r="S126" s="8"/>
       <c r="V126" s="9"/>
     </row>
-    <row r="127" spans="3:22" x14ac:dyDescent="0.25">
+    <row r="127" spans="2:22" x14ac:dyDescent="0.25">
       <c r="P127" s="8"/>
       <c r="Q127" s="8"/>
       <c r="S127" s="8"/>
       <c r="V127" s="9"/>
     </row>
-    <row r="128" spans="3:22" x14ac:dyDescent="0.25">
+    <row r="128" spans="2:22" x14ac:dyDescent="0.25">
       <c r="P128" s="8"/>
       <c r="Q128" s="8"/>
       <c r="S128" s="8"/>

</xml_diff>